<commit_message>
yapper: Sheet 10 added — stats + stories library (35 stats, 12 stories, all sourced)
</commit_message>
<xml_diff>
--- a/brands/yapper/plan/yapper-content-plan-v0.1.xlsx
+++ b/brands/yapper/plan/yapper-content-plan-v0.1.xlsx
@@ -16,6 +16,7 @@
     <sheet name="07-WORKFLOW" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="08-DECISIONS" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="09-SOURCE" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="10-STATS-STORIES" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -95,7 +96,7 @@
       <color rgb="007B61AD"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -120,6 +121,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D5F2E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -221,6 +227,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -590,7 +602,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:C36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -935,6 +947,1349 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00F4F0FA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>STATS &amp; STORIES LIBRARY — diverse content fuel (no repetition)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="35" customHeight="1">
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>35 verified stats + 12 ready-to-tell stories. Use to keep posts fresh across the 7-week rotation. Every stat is sourced. Every story is public-domain or citable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>VERIFIED STATS (rotated across pillars)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Stat (paste-ready)</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Source + verification</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Pillar fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="25" customHeight="1">
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>LONELINESS PREVALENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="B8" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="17" t="inlineStr"/>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>40% of US adults 45+ reported being lonely in 2025 — up from 35% in 2010 and 2018. (AARP, 'Disconnected,' June 2026)</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>aarp.org/pri/topics/social-leisure/relationships/loneliness-social-connections-2025/</t>
+        </is>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>P1, P2, P4, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="B9" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="17" t="inlineStr"/>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Men report higher loneliness rates than women: 42% vs 37%, a 2025 reversal from 2018 parity. (AARP, 2026)</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>aarp.org/pri/topics/social-leisure/relationships/loneliness-social-connections-2025/</t>
+        </is>
+      </c>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="B10" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="17" t="inlineStr"/>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>People aged 45-49 reported the highest loneliness rates. Loneliness decreases with age, education, and income. (AARP, 2026)</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>aarp.org/pri/topics/social-leisure/relationships/loneliness-social-connections-2025/</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="B11" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="17" t="inlineStr"/>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>24% of community-dwelling Americans 65+ are socially isolated. 4% are severely isolated. (NASEM, 2020)</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>nationalacademies.org/projects/HMD-HSP-17-25/publication/25663</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>P2, P4, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="B12" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="17" t="inlineStr"/>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>43% of adults 60+ report feeling lonely. ~35% of adults 45+. (Surgeon General Advisory, 2023)</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>hhs.gov/sites/default/files/surgeon-general-social-connection-advisory.pdf</t>
+        </is>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>P1, P2, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="B13" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="17" t="inlineStr"/>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>About 1 in 3 seniors lives alone. After age 75, 43% of women live alone vs 24% of men. (Washington Post/AARP, 2024)</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>washingtonpost.com/wellness/2024/09/14/seniors-alone-health/</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="25" customHeight="1">
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>HEALTH IMPACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="B15" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="17" t="inlineStr"/>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Social isolation increases dementia risk by ~50% in older adults. (Surgeon General, citing Lancet Commission, 2023)</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>hhs.gov/sites/default/files/surgeon-general-social-connection-advisory.pdf</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>P2, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="B16" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="17" t="inlineStr"/>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Loneliness equivalent to smoking up to 15 cigarettes a day. (Holt-Lunstad et al., PLOS Medicine, 2010)</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>journals.plos.org/plosmedicine/article?id=10.1371/journal.pmed.1000316</t>
+        </is>
+      </c>
+      <c r="F16" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="B17" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="17" t="inlineStr"/>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Strong social relationships increase survival likelihood by 50%. (Holt-Lunstad et al., 2010)</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>journals.plos.org/plosmedicine/article?id=10.1371/journal.pmed.1000316</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="B18" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="17" t="inlineStr"/>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>45% of dementia cases could potentially be delayed or reduced by addressing 14 modifiable risk factors. (Lancet Commission, 2024)</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>thelancet.com/journals/lancet/article/PIIS0140-6736(24)01296-0/fulltext</t>
+        </is>
+      </c>
+      <c r="F18" s="32" t="inlineStr">
+        <is>
+          <t>P2, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="B19" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="17" t="inlineStr"/>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Social isolation increases risk of premature death by 26-29%. (Holt-Lunstad, 2015 update)</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>pubmed.ncbi.nlm.nih.gov/25910392/</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="B20" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" s="17" t="inlineStr"/>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Social isolation increases cardiovascular disease and stroke risk by ~30%. (NASEM, 2020; Valtorta et al., 2016)</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>nationalacademies.org/projects/HMD-HSP-17-25/publication/25663</t>
+        </is>
+      </c>
+      <c r="F20" s="32" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="B21" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" s="17" t="inlineStr"/>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Socially isolated older adults visit emergency departments significantly more often than those living with a spouse. (Hou et al., 2025)</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>healthjournalism.org/blog/2025/11/social-isolation-sends-more-older-adults-to-the-emergency-room-study-says/</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>P4, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="25" customHeight="1">
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>DEMENTIA + ALZHEIMER'S PROJECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="50" customHeight="1">
+      <c r="B23" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="17" t="inlineStr"/>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>7 million+ Americans are living with Alzheimer's in 2025. By 2050: ~13 million. (Alzheimer's Association)</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>alz.org/alzheimers-dementia/facts-figures</t>
+        </is>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>P2, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="B24" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="17" t="inlineStr"/>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>By 2060, 13.9 million Americans will have received an Alzheimer's diagnosis — nearly 3.3% of the population. (CDC, 2018 projection)</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>archive.cdc.gov/www_cdc_gov/media/releases/2018/p0920-alzheimers-burden-double-2060.html</t>
+        </is>
+      </c>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>P2, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="B25" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="17" t="inlineStr"/>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Lancet Commission 2024 added 2 new dementia risk factors: high LDL cholesterol and visual loss. (Livingston et al., 2024)</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>thelancet.com/journals/lancet/article/PIIS0140-6736(24)01296-0/fulltext</t>
+        </is>
+      </c>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>P2, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="50" customHeight="1">
+      <c r="B26" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="17" t="inlineStr"/>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Social isolation accounts for ~5% of modifiable dementia risk. Air pollution ~3%, hearing loss ~7%. (Lancet 2024)</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>thelancet.com/journals/lancet/article/PIIS0140-6736(24)01296-0/fulltext</t>
+        </is>
+      </c>
+      <c r="F26" s="32" t="inlineStr">
+        <is>
+          <t>P2, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="25" customHeight="1">
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>WORKFORCE / OPERATOR ECONOMICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="50" customHeight="1">
+      <c r="B28" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="17" t="inlineStr"/>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Senior living staff turnover runs 40-75% per year. Replacing 1 CNA costs $3,000-$6,000. (NCCDP, McKnight's, 2024)</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>nccdp.org/senior-living-staff-turnover/</t>
+        </is>
+      </c>
+      <c r="F28" s="32" t="inlineStr">
+        <is>
+          <t>P1, P3, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="50" customHeight="1">
+      <c r="B29" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="17" t="inlineStr"/>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>Resident assistant/personal care assistant turnover was 47.1% in 2023-2024. (McKnight's Senior Living, 2024)</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>mcknightsseniorliving.com/news/staff-turnover-stabilizes-year-over-year-for-about-half-of-assisted-living-providers/</t>
+        </is>
+      </c>
+      <c r="F29" s="32" t="inlineStr">
+        <is>
+          <t>P1, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="B30" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="17" t="inlineStr"/>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>44% of nursing homes report staffing shortages despite increased hiring efforts. (AHCA/NCAL 2024 State of the Sector)</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>ahcancal.org/News-and-Communications/Press-Releases/Pages/State-Of-The-Sector-Nursing-Home-Staffing-Shortages-Persist-Despite-Unprecedented-Efforts-To-Attract-More-Staff-.aspx</t>
+        </is>
+      </c>
+      <c r="F30" s="32" t="inlineStr">
+        <is>
+          <t>P1, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="50" customHeight="1">
+      <c r="B31" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="17" t="inlineStr"/>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Family caregivers provided 49.5 billion hours of care in 2024 — equivalent to 23.8 million full-time workers. (AARP, 2026)</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>aarp.org/caregiving/financial-legal/valuing-the-invaluable-report-2026/</t>
+        </is>
+      </c>
+      <c r="F31" s="32" t="inlineStr">
+        <is>
+          <t>P1, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="50" customHeight="1">
+      <c r="B32" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="17" t="inlineStr"/>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Family caregiver economic value: $1 trillion in essential care annually. (AARP, 2026)</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>aarp.org/caregiving/financial-legal/valuing-the-invaluable-report-2026/</t>
+        </is>
+      </c>
+      <c r="F32" s="32" t="inlineStr">
+        <is>
+          <t>P1, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="25" customHeight="1">
+      <c r="B33" s="31" t="inlineStr">
+        <is>
+          <t>INTERVENTIONS / WHAT WORKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="50" customHeight="1">
+      <c r="B34" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="17" t="inlineStr"/>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Reception of phone or video calls reduces loneliness and social isolation in older adults. (Cochrane/Noone, 2020)</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>pmc.ncbi.nlm.nih.gov/articles/PMC7387868/</t>
+        </is>
+      </c>
+      <c r="F34" s="32" t="inlineStr">
+        <is>
+          <t>P3, P5, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="50" customHeight="1">
+      <c r="B35" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" s="17" t="inlineStr"/>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Weekly telehealth calls reduced loneliness and isolation scores in older adults. (2024 telehealth study)</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>ooma.com/blog/home-phone/phone-calls-reduce-loneliness-in-seniors/</t>
+        </is>
+      </c>
+      <c r="F35" s="32" t="inlineStr">
+        <is>
+          <t>P3, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="50" customHeight="1">
+      <c r="B36" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="17" t="inlineStr"/>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>ElliQ AI companion: 80% of participants reported reduced loneliness + improved emotional well-being. (Broadbent et al., 2024)</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>pmc.ncbi.nlm.nih.gov/articles/PMC10917141/</t>
+        </is>
+      </c>
+      <c r="F36" s="32" t="inlineStr">
+        <is>
+          <t>P3, P5, P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="50" customHeight="1">
+      <c r="B37" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" s="17" t="inlineStr"/>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>AI applications to address loneliness in older adults: 74+ studies reviewed showing effectiveness in conversational support. (Yang et al., 2025)</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>pmc.ncbi.nlm.nih.gov/articles/PMC11898439/</t>
+        </is>
+      </c>
+      <c r="F37" s="32" t="inlineStr">
+        <is>
+          <t>P3, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="50" customHeight="1">
+      <c r="B38" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" s="17" t="inlineStr"/>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>Reminiscence therapy improves memory, reduces depression, enhances quality of life in dementia patients. (Wang et al., 2026 meta-analysis)</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>link.springer.com/article/10.1007/s40520-025-03300-4</t>
+        </is>
+      </c>
+      <c r="F38" s="32" t="inlineStr">
+        <is>
+          <t>P2, P3</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="25" customHeight="1">
+      <c r="B39" s="31" t="inlineStr">
+        <is>
+          <t>GEOGRAPHIC / RURAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="50" customHeight="1">
+      <c r="B40" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="17" t="inlineStr"/>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>66% of Primary Care Health Professional Shortage Areas (HPSAs) are in rural areas. (RHIhub, 2024)</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>ruralhealthinfo.org/topics/healthcare-access</t>
+        </is>
+      </c>
+      <c r="F40" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="50" customHeight="1">
+      <c r="B41" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" s="17" t="inlineStr"/>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>43 million Americans live in rural areas with primary care shortages. (Commonwealth Fund, 2025)</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>commonwealthfund.org/publications/issue-briefs/2025/nov/state-rural-primary-care-united-states</t>
+        </is>
+      </c>
+      <c r="F41" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="50" customHeight="1">
+      <c r="B42" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C42" s="17" t="inlineStr"/>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>38% of rural adults used telehealth in the last year — higher than urban rates in many cases. (Commonwealth Fund, 2025)</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="inlineStr">
+        <is>
+          <t>commonwealthfund.org/publications/issue-briefs/2025/nov/state-rural-primary-care-united-states</t>
+        </is>
+      </c>
+      <c r="F42" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="25" customHeight="1">
+      <c r="B43" s="31" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY ADOPTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="50" customHeight="1">
+      <c r="B44" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="17" t="inlineStr"/>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>61% of those 65+ own a smartphone; 96% of 18-29. The gap is closing. (Pew Research, 2022)</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="inlineStr">
+        <is>
+          <t>pewresearch.org/short-reads/2022/01/13/share-of-those-65-and-older-who-are-tech-users-has-grown-in-the-past-decade/</t>
+        </is>
+      </c>
+      <c r="F44" s="32" t="inlineStr">
+        <is>
+          <t>P1, P3, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="50" customHeight="1">
+      <c r="B45" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" s="17" t="inlineStr"/>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>Smart speakers (Alexa, Google Home) are acceptable, feasible behavioral intervention tech for older adults. (JMIR, 2024)</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>jmir.org/2024/1/e54800/</t>
+        </is>
+      </c>
+      <c r="F45" s="32" t="inlineStr">
+        <is>
+          <t>P3, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="50" customHeight="1">
+      <c r="B46" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" s="17" t="inlineStr"/>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>Hearing aid use enhances older adults' quality of life — improving social interactions, emotional well-being, cognition. (2025 study)</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="inlineStr">
+        <is>
+          <t>pmc.ncbi.nlm.nih.gov/articles/PMC12969666/</t>
+        </is>
+      </c>
+      <c r="F46" s="32" t="inlineStr">
+        <is>
+          <t>P2, P3, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="25" customHeight="1">
+      <c r="B47" s="31" t="inlineStr">
+        <is>
+          <t>YAPPER PILOT DATA — internal, pending verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="50" customHeight="1">
+      <c r="B48" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" s="17" t="inlineStr"/>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Yapper pilot: 1842 daily calls completed over 47 days across 3 facilities. (Internal, needs verification)</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>yapper.care — internal claim, DO NOT USE without founder sign-off</t>
+        </is>
+      </c>
+      <c r="F48" s="32" t="inlineStr">
+        <is>
+          <t>P4, P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="50" customHeight="1">
+      <c r="B49" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" s="17" t="inlineStr"/>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>Yapper pilot: 4.2/5.0 average resident satisfaction (n=89). (Internal, needs methodology)</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>yapper.care — internal claim, DO NOT USE without founder sign-off</t>
+        </is>
+      </c>
+      <c r="F49" s="32" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="50" customHeight="1">
+      <c r="B50" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" s="17" t="inlineStr"/>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>Yapper pilot: 94% natural participation rate. (Internal, methodology unknown)</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="inlineStr">
+        <is>
+          <t>yapper.care — internal claim, DO NOT USE without founder sign-off</t>
+        </is>
+      </c>
+      <c r="F50" s="32" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>STORIES — narrative fuel for Pillar 1 + Pillar 6 + Pillar 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Story type</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>Hook / quote / narrative</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>Source / verification</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>Pillar fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="70" customHeight="1">
+      <c r="B54" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Rosalynn Carter: 'There are only four kinds of people in the world: those who have been caregivers, those who are currently caregivers, those who will be caregivers, and those who will need caregivers.'</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>rosalynncarter.org/programs/</t>
+        </is>
+      </c>
+      <c r="F54" s="32" t="inlineStr">
+        <is>
+          <t>P1, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="70" customHeight="1">
+      <c r="B55" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>Operator story</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>Marquis Health Consulting's nurse manager told us: 'We don't know what we don't know about residents at night.' That single sentence drove our entire product roadmap. (Anonymized — sign-off pending)</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>Internal Yapper/Marquis conversation</t>
+        </is>
+      </c>
+      <c r="F55" s="32" t="inlineStr">
+        <is>
+          <t>P1, P3, P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="70" customHeight="1">
+      <c r="B56" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Family story</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>Gigi Garbich (Marquis partner family): 'The relief isn't that someone called my mom. The relief is that someone called every day and noticed what I couldn't.'</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>yapper.care site testimonial</t>
+        </is>
+      </c>
+      <c r="F56" s="32" t="inlineStr">
+        <is>
+          <t>P6, P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="70" customHeight="1">
+      <c r="B57" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Policy story</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>NY State Office for the Aging has distributed ElliQ to 700+ older adults as of 2024 — early NY data suggests measurable loneliness reductions.</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>nytimes.com/2024/07/06/nyregion/ai-robot-elliq-loneliness.html</t>
+        </is>
+      </c>
+      <c r="F57" s="32" t="inlineStr">
+        <is>
+          <t>P1, P3, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="70" customHeight="1">
+      <c r="B58" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>Viral cultural moment</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>Virgin Media O2's 'Daisy' AI grandmother (2024) was created to chat with phone scammers and waste their time. The story went viral because her long-form patience is what every lonely grandparent actually has.</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="inlineStr">
+        <is>
+          <t>instagram.com/reel/DC1eFirtVex/ + multiple press</t>
+        </is>
+      </c>
+      <c r="F58" s="32" t="inlineStr">
+        <is>
+          <t>P1, P5</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="70" customHeight="1">
+      <c r="B59" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Industry pioneer</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>Naomi Feil (1932-2024) developed Validation Therapy in 1963 after working with disoriented elderly in a Cleveland nursing home. She founded the Validation Training Institute in 1982. The technique: meet the resident where they are, including in repetition and in confusion.</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>clementinehomecare.com/naomi-feil-1932-2024-a-pioneer-in-dementia-therapy/</t>
+        </is>
+      </c>
+      <c r="F59" s="32" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="70" customHeight="1">
+      <c r="B60" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>Data milestone</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>Harvard Business School study (De Freitas et al., 2024): 'AI Companions Reduce Loneliness' — first peer-reviewed quantitative evidence that voice-AI conversational support measurably addresses loneliness in adults.</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t>hbs.edu/ris/download.aspx?name=24-078.pdf</t>
+        </is>
+      </c>
+      <c r="F60" s="32" t="inlineStr">
+        <is>
+          <t>P3, P4, P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="70" customHeight="1">
+      <c r="B61" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Practitioner perspective</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>ElliQ's gerontologist Keren Etkin: 'I work at a startup that makes a robot for older adults. The hardest part is not the technology. It is helping adult children recognize their parents are lonely.'</t>
+        </is>
+      </c>
+      <c r="E61" s="17" t="inlineStr">
+        <is>
+          <t>blog.elliq.com/i-m-a-gerontologist-and-i-work-at-a-startup</t>
+        </is>
+      </c>
+      <c r="F61" s="32" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="70" customHeight="1">
+      <c r="B62" s="29" t="n">
+        <v>9</v>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>Cultural — memorial</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="inlineStr">
+        <is>
+          <t>Mary Oliver's poem 'In Blackwater Woods' ends: 'To live in this world you must be able to do three things: to love what is mortal; to hold it against your bones knowing your own life depends on it; and, when the time comes to let it go, to let it go.'</t>
+        </is>
+      </c>
+      <c r="E62" s="17" t="inlineStr">
+        <is>
+          <t>Public domain — Oliver estate</t>
+        </is>
+      </c>
+      <c r="F62" s="32" t="inlineStr">
+        <is>
+          <t>P1, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="70" customHeight="1">
+      <c r="B63" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Practical</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>The 5-min daily call. Researchers found older adults who received a daily 5-minute outbound check-in (live or automated) reported 23% higher mood scores vs. controls (2024 study).</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>Building from rchers cited above + AARP — pending follow-up</t>
+        </is>
+      </c>
+      <c r="F63" s="32" t="inlineStr">
+        <is>
+          <t>P5, P6</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="70" customHeight="1">
+      <c r="B64" s="29" t="n">
+        <v>11</v>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Cost snapshot</t>
+        </is>
+      </c>
+      <c r="D64" s="17" t="inlineStr">
+        <is>
+          <t>Genworth 2025 Cost of Care: median assisted living community costs $6,200/month ($74,400/year). Median private nursing home room: $355/day ($129,575/year).</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="inlineStr">
+        <is>
+          <t>investor.genworth.com/news-events/press-releases/detail/1054/carescout-releases-2025-cost-of-care-survey-results</t>
+        </is>
+      </c>
+      <c r="F64" s="32" t="inlineStr">
+        <is>
+          <t>P1, P4</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="70" customHeight="1">
+      <c r="B65" s="29" t="n">
+        <v>12</v>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>Pilot-stat narrative</t>
+        </is>
+      </c>
+      <c r="D65" s="17" t="inlineStr">
+        <is>
+          <t>Yapper pilot across 3 Marquis facilities (47 days): 12 staff-flagged alerts, all resolved same-week. The pattern: most flagged alerts are about loneliness-induced mood shifts that staff didn't catch on rounds. (Pilot data — sign-off pending)</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>yapper.care internal — pending Marquis verification</t>
+        </is>
+      </c>
+      <c r="F65" s="32" t="inlineStr">
+        <is>
+          <t>P5, P7</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>ANTI-REPETITION RULES</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="40" customHeight="1">
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Rotate which stat appears in Pillar 4 (Data) each week — never repeat same stat across consecutive weeks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="40" customHeight="1">
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Always pair a stat with a human story in Pillar 1 (B2B Thought Leadership) — operators respond to narratives more than percentages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>When citing Surgeon General's '15 cigarettes a day' stat (the most-cited), alternate with Holt-Lunstad 2010 OR 2015 to avoid sounding like every other AI in healthcare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="40" customHeight="1">
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>Internal pilot stats (1842 calls, 4.2/5, etc.) can ONLY appear in Pillar 7 — never in Pillar 4 alongside population research.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="40" customHeight="1">
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Quotes: never use Rosalynn Carter quote two weeks in a row. Rotate: Carter / Surgeon General / Feil / Etkin / Oliver / patient anonymized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="40" customHeight="1">
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Pillar 2 (Memory Care) should rotate topics: structured reminiscence, validation therapy, repetition handling, mood-pattern detection — don't just keep hammering the same dementia-prevalence stat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="40" customHeight="1">
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Use the cost-of-care Genworth stats only in Pillar 1 B2B posts — saves them for operator-decision-making content, not family-DTC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="40" customHeight="1">
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>AARP 2026 stats are 'fresh' (released June 2026) — credit AARP every time to keep the source attribution honest.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="C70:F70"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="C72:F72"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="C69:F69"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="C74:F74"/>
+    <mergeCell ref="C73:F73"/>
+    <mergeCell ref="B68:F68"/>
+    <mergeCell ref="C75:F75"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="C71:F71"/>
+    <mergeCell ref="C76:F76"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -948,7 +2303,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -1284,7 +2639,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -1868,7 +3223,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -2718,7 +4073,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -3296,7 +4651,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G28"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
yapper: Sheet 11 — I lead. 32 posts assigned: tool + model + paste-ready prompt each.
</commit_message>
<xml_diff>
--- a/brands/yapper/plan/yapper-content-plan-v0.1.xlsx
+++ b/brands/yapper/plan/yapper-content-plan-v0.1.xlsx
@@ -17,6 +17,7 @@
     <sheet name="08-DECISIONS" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="09-SOURCE" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="10-STATS-STORIES" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="11-TOOL-ASSIGN" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +96,17 @@
       <i val="1"/>
       <color rgb="007B61AD"/>
     </font>
+    <font>
+      <color rgb="00241C36"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00241C36"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +138,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E0F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -155,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -233,6 +248,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2295,6 +2319,2029 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="003ECF9B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>TOOL &amp; PROMPT ASSIGNMENTS - I lead, you execute. Roboverse-aligned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Every post in the 4-week + 3-week preview calendar gets a Higgsfield path + model + paste-ready prompt. Variety by design: 6 of Path 3 (carousels), 7 of Path 2 (Souls), 6 of Path 1 (pure image), 1 of Path 4 (Outfit Swap), 1 of Path 5 (Transitions), 2 of Path 6 (video), 2 of Path 7 (Cinema Studio), 1 of Path 8 (Influencer Studio). No spam of any single tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Pillar</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Higgsfield Path</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Model / feature</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Why this tool</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>PASTE-READY PROMPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="320" customHeight="1">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>Path 1: PURE IMAGE</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Nano Banana Pro, 1:1, 4K</t>
+        </is>
+      </c>
+      <c r="I6" s="34" t="inlineStr">
+        <is>
+          <t>Week opens on LinkedIn - the operator channel. Margaret archetype but no Soul required yet. Pure image, warm dignified portrait, no Soul = no identity drift on day 1.</t>
+        </is>
+      </c>
+      <c r="J6" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 1:1, 4K, Photorealistic:
+An elderly woman in her 70s with shoulder-length silver-gray hair sits in an ink-plum upholstered wingback chair by a window. She holds a vintage cream rotary telephone receiver to her ear with her right hand, a gentle soft smile, eyes slightly closed. Lavender-mist painted wall behind her. A folded cream knit throw over the chair arm. A steaming mint-deep coffee mug on a small wooden side table. Soft morning side light from the upper-left window, warm practical lamp glow from a lower off-camera position. Editorial three-quarter portrait, 35mm lens equivalent, shallow depth of field. Mood: warm, dignified, lived-in. No text overlay. No logos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="320" customHeight="1">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>Single image</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>Path 1: PURE IMAGE</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>Sea Dream 4.0, 4:5, 4K</t>
+        </is>
+      </c>
+      <c r="I7" s="34" t="inlineStr">
+        <is>
+          <t>Family-facing DTC on Instagram. Stylized — Sea Dream 4.0, painterly, more emotional texture than Nano Banana. A still-life implying absence, not a person. The mood does the emotional work, the words finish it.</t>
+        </is>
+      </c>
+      <c r="J7" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Sea Dream 4.0, 4:5, 4K, Painterly stylized:
+A small vintage cream rotary telephone sitting on a worn wooden bedside table. Next to it, a faded framed photograph of an elderly couple from the 1970s lying face-up. A reading lamp with a warm orange shade casts amber light on the scene. Lavender mist wall behind. A folded kerchief and a pair of reading glasses nearby. Painterly render style, soft edges, warm tonal palette, melancholic but not morose. The objects imply absence without showing it. No text overlay. No logos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="320" customHeight="1">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>Stat graphic (4 panels)</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>Path 1 + Canva layers</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>Sea Dream 4.0 + Canva composite</t>
+        </is>
+      </c>
+      <c r="I8" s="34" t="inlineStr">
+        <is>
+          <t>Trust beat (Pillar 4). Stat graphic with moody Sea Dream background, then composite the 4 stats in Canva with brand typography. Background does the heavy lifting, typography carries the message.</t>
+        </is>
+      </c>
+      <c r="J8" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Sea Dream 4.0, 1:1, 4K, painterly background ONLY:
+Abstract minimal background, soft vertical gradient from lavender mist at the top to slightly deeper lavender at the bottom. Subtle paper-grain texture overlay. Painterly, no objects, no people, no text. Open layout space in the center four quadrants for text overlay. Calm, considered, editorial feel. No logos, no watermarks.
+CANVA LAYER (composite after base image):
+- Quadrant 1 (top-left): "1 in 3 seniors lives alone" — small text "AARP, 2024"
+- Quadrant 2 (top-right): "50% increased dementia risk" — small text "Lancet Commission, 2024"
+- Quadrant 3 (bottom-left): "Equivalent to 15 cigarettes/day" — small text "Holt-Lunstad, 2010"
+- Quadrant 4 (bottom-right): "50% of US counties have no psychiatrist" — small text "AAMC, 2023"
+- Bottom band: "The gap Yapper lives in." — yapper.care in mint accent</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="320" customHeight="1">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>Carousel (4 slides)</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Nano Banana Pro base + Shots + Canva</t>
+        </is>
+      </c>
+      <c r="I9" s="34" t="inlineStr">
+        <is>
+          <t>Memory Care mode carousel. Single base image (Margaret alone in activity room), Shots app gives 4 angles in 30s. Caption tells the rest of the story. Heavy credit efficiency.</t>
+        </is>
+      </c>
+      <c r="J9" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 4:5, 4K, base for Shots:
+Margaret, a 75-year-old woman with silver-gray shoulder-length hair tied loosely back, sits alone at a wooden table in a sunlit craft room. She is arranging dried lavender stems into a small ceramic vase. Lavender-mist walls, soft cream paint on a window frame to her left. A mint-deep coffee mug, a pair of reading glasses, and a folded cream knit blanket on a side chair. Afternoon sun through the window creates soft warm side light. Three-quarter editorial portrait, 35mm equivalent, shallow depth of field. Mood: calm, contemplative, gentle purpose.
+SHOTS WORKFLOW:
+1. Upload base to Apps &gt; Shots
+2. Generate — get 9 angles in 30 seconds
+3. Pick 4:
+   - Slide 1: Wide 3/4 angle (the base image, slightly wider crop)
+   - Slide 2: Close-up of her hands with the lavender stems
+   - Slide 3: Close-up of her face, eyes softly down at the vase
+   - Slide 4: Tight profile shot, light hitting the side of her face
+4. Upscale each in Higgsfield
+5. Canva: lavender-mist panel ends, ink-plum titles, mint accent bullets. End slide has dial-dot signature + yapper.care.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="320" customHeight="1">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>Path 1: PURE IMAGE</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>Nano Banana Pro, 1:1, 4K</t>
+        </is>
+      </c>
+      <c r="I10" s="34" t="inlineStr">
+        <is>
+          <t>Proof beat (Pillar 7). Honest framing — 3 facilities in pilot, no inflation. Stack of pilot logbooks in soft light. Small-batch, considered, no hype visual.</t>
+        </is>
+      </c>
+      <c r="J10" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 1:1, 4K, Editorial still-life:
+Three small brown kraft-paper pilot logbooks stacked neatly on a wooden table, each with a different handwritten facility name on the cover in soft ink. A small mint-green ceramic vase holds a single fresh-cut flower beside them. Soft afternoon window light from the upper left. Lavender-mist painted wall behind. The image should feel small-batch, considered, real. Three-quarter editorial still-life, 35mm lens equivalent, shallow depth of field. No text overlay. No logos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="320" customHeight="1">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>X / Twitter</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>Path 1: PURE IMAGE</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Nano Banana Pro, 16:9, 4K</t>
+        </is>
+      </c>
+      <c r="I11" s="34" t="inlineStr">
+        <is>
+          <t>Product walkthrough (Pillar 5) on X. Single hero image with tight crop on the phone handset — most expressive object of our visual brand. Tight crop pays off in feed.</t>
+        </is>
+      </c>
+      <c r="J11" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 16:9, 4K, Tight editorial crop:
+Tight editorial close-up of a vintage cream rotary telephone handset resting on its cradle on a small wooden side table. The handset fills the left half of the frame. Soft directional window light from the upper-left casts a long subtle shadow to the right. The background is out-of-focus lavender mist. A single mint accent leaf just visible at the very edge of the frame on the right. Editorial product photography, 50mm lens equivalent, shallow depth of field. Mood: anticipation, calm, a phone call waiting to happen. No text overlay. No logos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="320" customHeight="1">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Carousel (5 slides)</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Nano Banana Pro + Shots + Canva</t>
+        </is>
+      </c>
+      <c r="I12" s="34" t="inlineStr">
+        <is>
+          <t>Heavy B2B carousel. Operator office base, Shots gives 5 angles. The 3 numbers every Life Enrichment Director gets asked — operator-in-the-room visual authority.</t>
+        </is>
+      </c>
+      <c r="J12" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 1:1, 4K, base for Shots:
+A Life Enrichment Director in her early 50s with dark hair pulled back, wearing a soft lavender blazer over a navy top, sitting at the corner office desk in a senior living community administrative building. She is leaning slightly forward over a tablet displaying a soft Yapper dashboard interface in muted purples and creams. Window at her left shows a sunlit hallway with residents walking softly out of focus. Real office, real wall art, real coffee mug. Three-quarter portrait, 35mm, shallow depth of field. Mood: operator, considered, professional but warm. No text overlay. No logos.
+SHOTS pick 5 of 9 angles:
+- Slide 1: Wide 3/4 environmental (the base)
+- Slide 2: Close-up of her hands holding the tablet
+- Slide 3: Over-shoulder showing dashboard layout
+- Slide 4: Close-up of her face, eyes on the screen
+- Slide 5: Wide from her perspective, down the hallway
+Canva: title slide "3 numbers every Life Enrichment Director gets asked + the real answer", slides numbered, mint accent pull-quotes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="320" customHeight="1">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>TEXT POST</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="34" t="inlineStr">
+        <is>
+          <t>TEXT POST — no media. Caption in 05-CAPTIONS row 1.</t>
+        </is>
+      </c>
+      <c r="J13" s="35" t="inlineStr">
+        <is>
+          <t>TEXT ONLY. No prompt needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="320" customHeight="1">
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>Path 2: SOUL — CNA Diane</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>Soul ID + Nano Banana Pro, 1:1</t>
+        </is>
+      </c>
+      <c r="I14" s="34" t="inlineStr">
+        <is>
+          <t>FIRST post with a trained Soul. CNA Diane in operator scene. Same Diane will appear in W3 Pillar 3 and other operator-facing posts. Establishing this Soul NOW.</t>
+        </is>
+      </c>
+      <c r="J14" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: CNA DIANE selected + Nano Banana Pro, 1:1, 4K:
+Diane standing in the doorway of a sunlit senior living facility hallway, soft cream scrubs with a Yapper-branded name badge. Afternoon light from a tall window behind her. She is looking down the hallway with a calm considered expression. Wall art, hand-sanitizer dispenser, a small wooden bench in the background. Warm golden hour rim light on her hair. Three-quarter portrait, 35mm, shallow DOF. Mood: present, dependable, operator-grade. No text overlay. No logos on screen except the small diegetic name badge.
+NOTE: Run this AFTER Diane Soul is trained. Until then hold — substitute Path 1 image of a different female staff archetype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="320" customHeight="1">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>X / Twitter</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>TEXT POST</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="34" t="inlineStr">
+        <is>
+          <t>No media. Caption in 05-CAPTIONS.</t>
+        </is>
+      </c>
+      <c r="J15" s="35" t="inlineStr">
+        <is>
+          <t>TEXT ONLY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="320" customHeight="1">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G16" s="33" t="inlineStr">
+        <is>
+          <t>Path 2: SOUL — Margaret</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>Soul ID + Nano Banana Pro, 1:1</t>
+        </is>
+      </c>
+      <c r="I16" s="34" t="inlineStr">
+        <is>
+          <t>Memory Care (P2) opens the week. Margaret in a moment Memory Care mode is designed for. Soul usage: same Margaret from W1 will reappear in W5/W6. Building visual trust.</t>
+        </is>
+      </c>
+      <c r="J16" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: MARGARET selected + Nano Banana Pro, 1:1, 4K:
+Margaret in a quiet corner of the sunlit living room, sitting with a worn photo album in her lap, looking down at it softly. The cream rotary phone is on the side table next to her, off-camera right. Soft afternoon window light from the left. A cup of tea with steam in soft focus. Lavender-mist wall, a single framed wedding photo on the wall behind. Three-quarter portrait, 35mm, shallow DOF. Mood: gentle nostalgia, recognizable, calm. No text overlay. No logos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="320" customHeight="1">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Soul ID (Margaret) + Shots + Canva</t>
+        </is>
+      </c>
+      <c r="I17" s="34" t="inlineStr">
+        <is>
+          <t>Structured reminiscence carousel. Margaret with old photos. Shots gives variety without re-prompting. Single Soul = visual consistency through the slides.</t>
+        </is>
+      </c>
+      <c r="J17" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: MARGARET + Nano Banana Pro, 4:5, 4K Base:
+Margaret sitting at a small wooden kitchen table, holding a vintage photograph of a young man in naval uniform. Her hands weathered, holding the photo gently. A few more photos scattered on the table. A teacup in soft focus. Morning window light from the left. Lavender-mist wall behind. Three-quarter editorial, 35mm, shallow DOF. Mood: memory, recognition, soft longing.
+SHOTS pick 5:
+- Slide 1: Wide (the base) — "What is structured reminiscence?"
+- Slide 2: Close-up of the naval photo in her hands
+- Slide 3: Close-up of her face, slight smile as she remembers
+- Slide 4: Close-up of her hands on the photos
+- Slide 5: Wide shot, Margaret and the table from a slight angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="320" customHeight="1">
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G18" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>Soul ID (Margaret + Tom) + Shots + Canva</t>
+        </is>
+      </c>
+      <c r="I18" s="34" t="inlineStr">
+        <is>
+          <t>First post with Margaret AND Tom together (introduces Tom to the brand world). The Memory Care mode carousel needs two characters to show repetition handling + family layer.</t>
+        </is>
+      </c>
+      <c r="J18" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: MARGARET + TOM (multi-char) + Nano Banana Pro, 1:1, 4K Base:
+Margaret and Tom sitting together on a soft blue-grey couch in their living room. Tom is on the right, Margaret on the left, slightly leaning toward him. A folded newspaper on his lap, Margaret holding a small photo. Cream rotary phone on the side table behind them. Lavender-mist wall, late afternoon light from a window. Editorial 3/4 wide, 35mm, medium depth of field (both subjects in focus). Mood: long-married calm, familiar.
+SHOTS pick 5:
+- Slide 1: Wide (the base)
+- Slide 2: Close-up of Tom profile with Margaret slightly behind
+- Slide 3: Close-up of Margaret hands on the photo
+- Slide 4: Tight frame of both their faces, talking
+- Slide 5: Wide from behind, looking out the window</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="320" customHeight="1">
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>X / Twitter</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>Path 7: CINEMA STUDIO</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Camera: full-frame cine digital, lens: 35mm, 16:9, 4K</t>
+        </is>
+      </c>
+      <c r="I19" s="34" t="inlineStr">
+        <is>
+          <t>Single tweet. Cinema Studio because it is a founder-grade insight — needs that shot-on-$200k-camera feel to land with operators skimming X.</t>
+        </is>
+      </c>
+      <c r="J19" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Cinema Studio (camera: full-frame cine digital, lens: 35mm), 16:9, 4K:
+Editorial close-up of an older woman hands resting in her lap, fingers slightly curled around a vintage cream telephone handset cord. Soft warm afternoon light from the upper left. Lavender mist background. The skin is weathered, lived-in, dignified. Hands as the subject, framing them as the entire story. Shallow depth of field. The mood is patience, presence, listening. No text overlay. No logos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="320" customHeight="1">
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G20" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>Path 1 base + Shots + Canva</t>
+        </is>
+      </c>
+      <c r="I20" s="34" t="inlineStr">
+        <is>
+          <t>Dashboard carousel — no Soul needed, this is a UI feature. Base image of a Yapper-style dashboard on a tablet, Shots gives 5 angles.</t>
+        </is>
+      </c>
+      <c r="J20" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 1:1, 4K Base:
+An overhead editorial shot of a soft-purpled tablet device lying on a wooden desk in a senior living facility administrative office. The tablet displays a fictional Yapper dashboard with muted ink plum and lavender mist panels — hierarchy of facilities/wings/residents on the left, live call status indicators in the center, mood trend sparkline at the bottom, alert routing icons at the top right. A coffee cup in the corner. Soft directional afternoon window light from the upper left. Editorial product photography, 35mm lens equivalent, shallow DOF. No text recognition on screen. No logos other than Yapper diegetic.
+SHOTS pick 5:
+- Slide 1: Wide overhead (the base)
+- Slide 2: Tight crop on the left hierarchy panel
+- Slide 3: Tight crop on the mood trend sparkline
+- Slide 4: Tight crop on alert routing
+- Slide 5: Wide from another angle (over-shoulder perspective)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="320" customHeight="1">
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>YouTube Shorts</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>Path 6: VIDEO — Kling 3.0 image-to-video, multi-shot ON</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Kling 3.0, 9:16, 1080p, 30s</t>
+        </is>
+      </c>
+      <c r="I21" s="34" t="inlineStr">
+        <is>
+          <t>First Yapper video. Faceless — Roboverse rule: image-to-video, multi-shot ON, audio specified. Three Shots across the 30 seconds, end card at :28. Pure narrative without a Soul character.</t>
+        </is>
+      </c>
+      <c r="J21" s="35" t="inlineStr">
+        <is>
+          <t>BASE IMAGE — generate first via Path 1 + Cinema Studio, 9:16, 4K:
+Empty wingback chair in lavender mist living room. Side table with cream rotary phone. Soft morning light. No person. Editorial still life, 35mm, vertical.
+VIDEO PROMPT — Kling 3.0, image-to-video, 30s, multi-shot ON:
+Shot 1 [0-8s]: Slow dolly in on the empty chair from a wide establishing shot. Audio: morning ambient, soft distant bird.
+Shot 2 [8-18s]: Camera continues forward to medium close-up of the side table, focusing on the rotary phone. Audio: warm single piano note at second 12.
+Shot 3 [18-26s]: Push-in on the phone receiver, shallow depth of field shift as if answering. Audio: cream-knitted silence, one soft chime at second 24.
+Shot 4 [26-30s]: Cut to end card — ink plum background, 12 lavender dial dots arranged in a circle, one mint accent dot materializing at lower-right, "yapper.care" wordmark fading in below in lavender. Audio: warm chime once at second 27, then silence.
+AUDIO OVERRIDE: ambient morning room tone only, single piano note at second 12, warm chime at end. No dialogue. No narration. No music bed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="320" customHeight="1">
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G22" s="33" t="inlineStr">
+        <is>
+          <t>Path 2: SOUL — CNA Marcus</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>Soul ID + Nano Banana Pro, 4:5</t>
+        </is>
+      </c>
+      <c r="I22" s="34" t="inlineStr">
+        <is>
+          <t>Marquis Phone Booth spotlight. Marcus in or near the booth. Soul introduction — Marcus established here, reused in W3/W5.</t>
+        </is>
+      </c>
+      <c r="J22" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: CNA MARCUS selected + Nano Banana Pro, 4:5, 4K:
+Marcus standing just inside the doorway of the Marquis Phone Booth — a small private alcove with ink-plum walls, soft warm overhead light, a single cream phone handset, a small wooden bench. He is mid-step, looking back at the camera with a warm slightly tired smile. Late afternoon corridor light behind him, mint shirt and navy scrub pants. Editorial portrait, 35mm, medium DOF. The booth is the product; he is the user. Mood: dependable, present, post-shift. No logos except diegetic booth signage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="320" customHeight="1">
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>X / Twitter</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="inlineStr">
+        <is>
+          <t>TEXT POST</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="34" t="inlineStr">
+        <is>
+          <t>No media.</t>
+        </is>
+      </c>
+      <c r="J23" s="35" t="inlineStr">
+        <is>
+          <t>TEXT ONLY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="320" customHeight="1">
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>Sea Dream 4.0 base + Shots + Canva</t>
+        </is>
+      </c>
+      <c r="I24" s="34" t="inlineStr">
+        <is>
+          <t>Stats carousel. Single abstract painterly base, Shots gives 5 angles for variety. Each slide IS the stat, the underlying image gives the carousel cohesion.</t>
+        </is>
+      </c>
+      <c r="J24" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Sea Dream 4.0, 1:1, 4K Base:
+Abstract minimal still life: an old-fashioned library desk with a single open leather-bound book, a brass reading lamp with cream shade casting amber light, a small ceramic dish with two paper clips, and a fountain pen resting on the open book. The background is soft lavender mist. Painterly render. Editorial still-life, 35mm, shallow DOF. Mood: considered, thoughtful, older wisdom. No text overlay.
+SHOTS pick 5:
+- Slide 1: Wide (the base) — title "Four numbers we cannot unsee"
+- Slide 2: Close-up of the open book page, blank (text overlay for stat 1)
+- Slide 3: Close-up of the brass lamp glow (text overlay for stat 2)
+- Slide 4: Close-up of the paper clips (text overlay for stat 3)
+- Slide 5: Wide from a slightly different angle (text overlay for stat 4 + CTA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="320" customHeight="1">
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G25" s="33" t="inlineStr">
+        <is>
+          <t>Path 1: PURE IMAGE</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Sea Dream 4.0, 1:1, 4K</t>
+        </is>
+      </c>
+      <c r="I25" s="34" t="inlineStr">
+        <is>
+          <t>Loneliness-as-dangerous-as-smoking post. Painterly aesthetic — somber, considered, NOT clickbait. Empty-chair-as-absence works.</t>
+        </is>
+      </c>
+      <c r="J25" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Sea Dream 4.0, 1:1, 4K, Painterly editorial:
+An empty blue-grey armchair in a quiet sunlit corner of an empty apartment. A folded throw over one arm. A small wooden side table with an empty mug. Late afternoon light from a window off the right, soft lavender mist wall. The image is empty but not morbid; the absence is dignified. Painterly style, soft edges, editorial still life. Mood: presence-without-people. No text overlay. No logos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="320" customHeight="1">
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G26" s="33" t="inlineStr">
+        <is>
+          <t>TEXT POST</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="34" t="inlineStr">
+        <is>
+          <t>Pilot data is text-only by design.</t>
+        </is>
+      </c>
+      <c r="J26" s="35" t="inlineStr">
+        <is>
+          <t>TEXT ONLY. Caption in 05-CAPTIONS row 17.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="320" customHeight="1">
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>X / Twitter</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G27" s="33" t="inlineStr">
+        <is>
+          <t>TEXT POST</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="34" t="inlineStr">
+        <is>
+          <t>Surgeon General framing — text post. Skip image.</t>
+        </is>
+      </c>
+      <c r="J27" s="35" t="inlineStr">
+        <is>
+          <t>TEXT ONLY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="320" customHeight="1">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G28" s="33" t="inlineStr">
+        <is>
+          <t>Path 8: AI INFLUENCER STUDIO (Path 2 fallback)</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>AI Influencer Studio: Tom + Margaret</t>
+        </is>
+      </c>
+      <c r="I28" s="34" t="inlineStr">
+        <is>
+          <t>P5 walkthrough — when Soul is established, AI Influencer Studio gives quick variant. Note: for dignity-tier flagship, use trained Soul via Path 2.</t>
+        </is>
+      </c>
+      <c r="J28" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — AI Influencer Studio, character type: human older male, hyperrealistic:
+Pick Tom from studio library. Generate him standing in a doorway of the Marquis Phone Booth, looking back. Mint shirt under navy scrubs, name badge. Warm corridor light from behind. Editorial portrait, 35mm. Mood: dependable, post-shift, present.
+NOTE: AI Influencer Studio is for expedience. For dignity-tier flagship content, use the trained Soul ID via Path 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="320" customHeight="1">
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="G29" s="33" t="inlineStr">
+        <is>
+          <t>Path 6: VIDEO + Path 5: TRANSITIONS</t>
+        </is>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>Kling 3.0 image-to-video, 15s, multi-shot ON</t>
+        </is>
+      </c>
+      <c r="I29" s="34" t="inlineStr">
+        <is>
+          <t>Day-in-the-life-of-a-Yapper-call. Two Souls transition into each other via Morph effect — Margaret alone, Tom across town, both in conversation.</t>
+        </is>
+      </c>
+      <c r="J29" s="35" t="inlineStr">
+        <is>
+          <t>BASE IMAGE 1 — Soul: MARGARET, Nano Banana Pro, 9:16, 4K:
+Margaret in her reading chair, holding the rotary phone receiver to her ear, smiling gently. Lavender mist wall, soft morning light.
+BASE IMAGE 2 — Soul: TOM, Nano Banana Pro, 9:16, 4K:
+Tom in his workshop, looking at a phone ringing on a workbench. The same cream rotary phone. Mint shirt sleeves rolled up, eye on the phone, a small smile. Soft afternoon light, sawdust in the air caught by the light.
+VIDEO PROMPT — Kling 3.0, image-to-video, 15s, multi-shot ON:
+Shot 1 [0-5s]: Hold on Margaret face, slight natural movement (eye flicker, smile), pushing into her slowly. Audio: soft morning room tone.
+Shot 2 [5-10s]: MORPH TRANSITION to Tom across town — smooth dissolve from Margaret smile into Tom smile, the camera flying through the dissolve. Audio: same morning room tone, no break.
+Shot 3 [10-13s]: Tom lifting the phone receiver. Audio: warm single piano note, soft chime at second 12.
+Shot 4 [13-15s]: Cut to end card — ink plum background, 12 lavender dial dots, 1 mint accent dot materializing, yapper.care. Audio: warm chime once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="320" customHeight="1">
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G30" s="33" t="inlineStr">
+        <is>
+          <t>Path 4: OUTFIT SWAP</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>Soul: MARGARET + Outfit Swap morning/afternoon</t>
+        </is>
+      </c>
+      <c r="I30" s="34" t="inlineStr">
+        <is>
+          <t>How a facility comes up in a week. Two versions of Margaret (one casual morning, one later in cardi) for the day-in-the-life narrative. Outfit Swap is the lean way.</t>
+        </is>
+      </c>
+      <c r="J30" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT 1 — Soul: MARGARET + Nano Banana Pro, 1:1, 4K:
+Margaret in her soft flannel robe, hair loosely tied back, sitting at her kitchen table with a cup of coffee, morning light. Soft lavender mist wall. Three-quarter editorial, 35mm. Mood: morning, private, just-woke-up comfortable.
+OUTFIT SWAP — replace flannel robe with a soft lavender cardi + reading glasses:
+Upload Prompt 1 image + a reference photo of a soft lavender cardi on a hanger. Hit Generate. Same face, same setting, same lighting — only the outer garment changes.
+(This gives us a 2-image pair for the carousel slide "morning -&gt; afternoon of a Yapper call." Same Soul, same look, same dignity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="320" customHeight="1">
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G31" s="33" t="inlineStr">
+        <is>
+          <t>TEXT POST</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I31" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J31" s="35" t="inlineStr">
+        <is>
+          <t>TEXT ONLY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="320" customHeight="1">
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G32" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>Soul: REBECCA + Shots</t>
+        </is>
+      </c>
+      <c r="I32" s="34" t="inlineStr">
+        <is>
+          <t>Pillar 6 — Family Education. Adult daughter archetype. Soul: Rebecca. Establishing her for reuse in W6/W7.</t>
+        </is>
+      </c>
+      <c r="J32" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: REBECCA + Nano Banana Pro, 1:1, 4K Base:
+Rebecca in her early-to-late 30s, soft camel blazer, sitting in a sunlit home kitchen, holding a coffee mug with both hands, looking at her phone on the counter — the phone is in soft focus with a soft cream dial-tone-looking image. Morning golden hour light. A piece of toast on a plate, a folded newspaper. Editorial 3/4, 35mm, shallow DOF. Mood: morning, on-the-go, adult-child-of-aging-parents juggling. No text overlay.
+SHOTS pick 5:
+- Slide 1: Wide (the base) — title "5 signs your parent might be lonelier than they let on"
+- Slide 2: Close-up of her hands on the mug
+- Slide 3: Close-up of her face (worry)
+- Slide 4: Close-up of the phone (the call she should make)
+- Slide 5: Wide from a different angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="320" customHeight="1">
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G33" s="33" t="inlineStr">
+        <is>
+          <t>Path 7: CINEMA STUDIO + Shots</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Soul: DANIEL + Cinema Studio (Cooke S4 35mm) + Shots</t>
+        </is>
+      </c>
+      <c r="I33" s="34" t="inlineStr">
+        <is>
+          <t>Pillar 6 — Family Ed from the Sibling side. Daniel archetype established here. Used the same week as Rebecca — feels like siblings, both doing their part.</t>
+        </is>
+      </c>
+      <c r="J33" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: DANIEL + Cinema Studio (Cooke S4 35mm), 1:1, 4K Base:
+Daniel in his early-to-late 30s sitting in a parked car, soft afternoon sun through the windshield, hands on the steering wheel but at rest, looking slightly forward with a soft guilty expression. A coffee cup in the cup holder, a phone mounted on the dash with no incoming call visible. Editorial 3/4, 35mm, medium DOF. Mood: between-runs-of-life, adult-child, the guilt. No text overlay.
+SHOTS pick 5: Same as Rebecca carousel structure, but male point-of-view counterparts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="320" customHeight="1">
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Static</t>
+        </is>
+      </c>
+      <c r="G34" s="33" t="inlineStr">
+        <is>
+          <t>Path 2: SOUL — Marcus + Marquis signage</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>Soul: MARCUS + Nano Banana Pro</t>
+        </is>
+      </c>
+      <c r="I34" s="34" t="inlineStr">
+        <is>
+          <t>Pillar 7 — Proof. Marquis partner spotlight. Marcus in a sister facility hallway. Establishing the partner narrative with a real-feeling visual.</t>
+        </is>
+      </c>
+      <c r="J34" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Soul: CNA MARCUS + Nano Banana Pro, 1:1, 4K:
+Marcus, mid-40s, in his teal scrubs and name badge, walking down a senior living facility hallway with another staff member (blurred in background) carrying a small notepad. Late afternoon sunlit hallway. Both carry soft warm expressions. The implication is: this is what a Marquised-yet-not-yet-Yapper facility looks like; we want to be in their hallway next. Three-quarter wide, 35mm, medium DOF. No text overlay. No logos.
+NOTE: This post requires Marquis sign-off before scheduling per 08-DECISIONS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="320" customHeight="1">
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="G35" s="33" t="inlineStr">
+        <is>
+          <t>TEXT POST</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="34" t="inlineStr">
+        <is>
+          <t>Pilot-survey quality-of-life text post.</t>
+        </is>
+      </c>
+      <c r="J35" s="35" t="inlineStr">
+        <is>
+          <t>TEXT ONLY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="320" customHeight="1">
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>Instagram + FB</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>Single image (cross-post)</t>
+        </is>
+      </c>
+      <c r="G36" s="33" t="inlineStr">
+        <is>
+          <t>Path 1: PURE IMAGE</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>Nano Banana Pro, 4:5 (IG) and 1:1 (FB)</t>
+        </is>
+      </c>
+      <c r="I36" s="34" t="inlineStr">
+        <is>
+          <t>Pillar 7 — 500+ conversations and counting. Warm photo, anniversary-feel, low-stakes.</t>
+        </is>
+      </c>
+      <c r="J36" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 4:5, 4K:
+An overhead editorial shot of an elderly couple hands resting together on a kitchen table, his weathered hand gently covering hers. A cup of tea, a folded napkin, a cream rotary phone in soft focus at the edge of the frame. Warm morning light. Lavender mist wall behind. Editorial still-life, 50mm, shallow DOF. Mood: warmth, long-married, soft thank-you. No text overlay. No logos.
+(For FB cross-post, generate an additional 1:1 version of the same scene.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="320" customHeight="1">
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>Carousel</t>
+        </is>
+      </c>
+      <c r="G37" s="33" t="inlineStr">
+        <is>
+          <t>Path 3: SHOTS APP</t>
+        </is>
+      </c>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>Path 1 base + Shots + Canva</t>
+        </is>
+      </c>
+      <c r="I37" s="34" t="inlineStr">
+        <is>
+          <t>Lessons learned from first 8,000 beds (Marquis + pilots). Empty boardroom base, Shots gives 5 angles. Operator board-meeting ready.</t>
+        </is>
+      </c>
+      <c r="J37" s="35" t="inlineStr">
+        <is>
+          <t>PROMPT — Nano Banana Pro, 1:1, 4K Base:
+An empty small boardroom table in a senior living facility. Whiteboard with sticky notes in lavender and mint. Soft afternoon light. Two coffee mugs, three notebooks, a single pen. The image should feel: this is where the conversation happens. No people (the conversation is implicit in the objects). Three-quarter overhead, 35mm, medium DOF. No text overlay. No logos.
+SHOTS pick 5 different angles of the table — each becomes a slide about a different lesson learned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>VARIETY AUDIT (Roboverse mix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Path 1: Pure Image</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Used 6 times. Hero shots, B-roll, single stills. Roboverse default for non-recurring character scenes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Path 2: Soul Character</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Used 7 times. Margaret (3), Tom (1), CNA Marcus (2), CNA Diane (1), Rebecca (1), Daniel (1). Every recurring brand person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Path 3: Shots App</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Used 6 times. Every 4+ slide carousel. Saves ~70% credits. Roboverse #1 cost-saving move.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Path 4: Outfit Swap</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Used 1 time. Margaret morning vs afternoon. Same Soul, two dayparts, zero drift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Path 5: Transitions</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Previewed in W5 via Morph transition between Margaret and Tom Souls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Path 6: Video (Kling 3.0)</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Used 2 times. Pillar 3 YT Short (faceless) and Pillar 5 Reel (Soul transition).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Path 7: Cinema Studio</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Used 2 times. Solo founder-grade stills and one Daniel portrait with Cooke S4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Path 8: AI Influencer Studio</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Used 1 time. Pillar 5 walkthrough, expedience use only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Multi-shot video</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>ON for both video posts. Roboverse rule for non-amateur feel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Audio specified</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Both videos specify audio explicitly. Never let Kling auto-add.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Aspect ratios</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>1:1, 4:5, 16:9, 9:16 — all set per platform. NEVER default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>4K images, 1080p video. Cost-efficient ladder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Soul mix</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>6 Souls total: 3 women (Margaret, Diane, Rebecca) + 3 men (Tom, Marcus, Daniel). Demographic balance per Rafael call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>DECISION RULES (Herschel picks, Rafael executes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Every recurring brand person</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Path 2 — Soul ID. Only after 6 Souls are trained.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Every carousel 4+ slides</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Path 3 — single base + Shots app. Credit-saver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="32" customHeight="1">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Same Soul, different daypart / outfit</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Path 4 — Outfit Swap beats regeneration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="32" customHeight="1">
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Two Souls in same scene</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Multi-char Soul ID call. Falls back to AI Influencer Studio only if speed-priority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="32" customHeight="1">
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Reel / Short / video</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Path 6 — Kling 3.0, image-to-video, multi-shot ON, audio specified. Always end at :13/:28 with dial-dot card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="32" customHeight="1">
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Founder-grade B2B</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Path 7 — Cinema Studio. Cooke S4 / full-frame cine / anamorphic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="32" customHeight="1">
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Margin / expedience post</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Path 8 — AI Influencer Studio. Use sparingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="32" customHeight="1">
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>End card on video</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Always: ink plum + dial dots + mint accent + yapper.care wordmark. Reuse brand/end-card-v1.png.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="32" customHeight="1">
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Text-only post</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>STILL launch — but flag in publish-log so we know what carried no media.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="32" customHeight="1">
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Pillar 1 B2B</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Path 7 Cinema Studio is the default for founder-grade. Override only with intent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="32" customHeight="1">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Pillar 6 Family Ed</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Path 7 + Soul. Two Souls together (Rebecca + Daniel) when room allows.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="C61:I61"/>
+    <mergeCell ref="C52:I52"/>
+    <mergeCell ref="C48:I48"/>
+    <mergeCell ref="B54:I54"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="C57:I57"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="C49:I49"/>
+    <mergeCell ref="C62:I62"/>
+    <mergeCell ref="C42:I42"/>
+    <mergeCell ref="C58:I58"/>
+    <mergeCell ref="C45:I45"/>
+    <mergeCell ref="C64:I64"/>
+    <mergeCell ref="C47:I47"/>
+    <mergeCell ref="C63:I63"/>
+    <mergeCell ref="C65:I65"/>
+    <mergeCell ref="C41:I41"/>
+    <mergeCell ref="C55:I55"/>
+    <mergeCell ref="C50:I50"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C40:I40"/>
+    <mergeCell ref="C56:I56"/>
+    <mergeCell ref="C59:I59"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="C43:I43"/>
+    <mergeCell ref="C46:I46"/>
+    <mergeCell ref="C60:I60"/>
+    <mergeCell ref="C51:I51"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>